<commit_message>
fix: rename export to export-excel and remove conflicting directory
</commit_message>
<xml_diff>
--- a/LISTAS DE BUENA FE AFA SOMOS TODOS 2026/BOCA 1.xlsx
+++ b/LISTAS DE BUENA FE AFA SOMOS TODOS 2026/BOCA 1.xlsx
@@ -276,515 +276,6 @@
   </cellStyles>
   <dxfs count="0"/>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer">
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>1781175</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>885825</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="981075" cy="904875"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image18.jpg"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>38100</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="904875" cy="819150"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image5.jpg"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>1152525</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="1076325" cy="1143000"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image15.jpg"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId3"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="1057275" cy="657225"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image3.jpg"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId4"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="1057275" cy="1019175"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image2.jpg"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId5"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="1000125" cy="1066800"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image1.jpg"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId6"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="438150" cy="990600"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image17.jpg"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId7"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="600075" cy="971550"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image4.jpg"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId8"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="828675" cy="1143000"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image16.jpg"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId9"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="542925" cy="1095375"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image10.jpg"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId10"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="590550" cy="1009650"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image7.jpg"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId11"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>13</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="666750" cy="1162050"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image9.jpg"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId12"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="561975" cy="952500"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image13.jpg"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId13"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="476250" cy="876300"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image6.jpg"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId14"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="1057275" cy="914400"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image8.jpg"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId15"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="1057275" cy="914400"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image14.jpg"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId16"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="1057275" cy="1104900"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image12.jpg"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId17"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="1057275" cy="1104900"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image11.jpg"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId18"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>